<commit_message>
Correction of "TEK Warmwasser" for usage "Wohnen"
Correction of TEK Warmwasser for usage Wohnen, Wohnen EFH and Wohnen MFH.
</commit_message>
<xml_diff>
--- a/src/dibs_data/data/auxiliary/TEKs/TEK_NWG_Vergleichswerte.xlsx
+++ b/src/dibs_data/data/auxiliary/TEKs/TEK_NWG_Vergleichswerte.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\André\Documents\Sicherung von altem NB\Documents\10_Projekte\2023_LEZBau\DIBS Wohnen\TEKs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\André\Documents\GitHub\DibsData\src\dibs_data\data\auxiliary\TEKs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B7F979F-83F6-4EBD-951F-ADF0A5984461}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FFC371-E08E-4631-B19E-5C654DE9DB6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TEK_Vergl_NWG" sheetId="1" r:id="rId1"/>
@@ -1311,12 +1311,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="129.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="141" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -1380,7 +1380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
@@ -1412,7 +1412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>12</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>14</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>16</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>23</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>24</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>25</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>26</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>27</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>28</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>29</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>30</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>31</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>32</v>
       </c>
@@ -2084,7 +2084,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -2116,7 +2116,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>34</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>35</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>36</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>37</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>38</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>39</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>40</v>
       </c>
@@ -2340,7 +2340,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>41</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>42</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>43</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>44</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>45</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>46</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>47</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>48</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>49</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>50</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>51</v>
       </c>
@@ -2692,7 +2692,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>52</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>53</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>54</v>
       </c>
@@ -2788,7 +2788,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>55</v>
       </c>
@@ -2820,7 +2820,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>56</v>
       </c>
@@ -2852,7 +2852,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>57</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>58</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>59</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>60</v>
       </c>
@@ -2980,7 +2980,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
         <v>61</v>
       </c>
@@ -3012,7 +3012,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="16" t="s">
         <v>71</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="16" t="s">
         <v>76</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="16" t="s">
         <v>157</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="16" t="s">
         <v>75</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="16" t="s">
         <v>77</v>
       </c>
@@ -3188,34 +3188,34 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="28" t="s">
         <v>175</v>
       </c>
       <c r="C59" s="28">
-        <v>25</v>
+        <v>12.5</v>
       </c>
       <c r="J59" s="13">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="28" t="s">
         <v>176</v>
       </c>
       <c r="C60" s="28">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J60" s="13">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="28" t="s">
         <v>178</v>
       </c>
       <c r="C61" s="28">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="J61" s="14">
         <v>60</v>
@@ -3231,14 +3231,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA552F24-7F73-483F-9F61-9FA1662119AB}">
   <dimension ref="A1:XFD122"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.5546875" customWidth="1"/>
-    <col min="2" max="2" width="116.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.5703125" customWidth="1"/>
+    <col min="2" max="2" width="116.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16384" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16384" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>63</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>65</v>
       </c>
@@ -3257,7 +3257,7 @@
       <c r="C2" s="23"/>
       <c r="D2" s="20"/>
     </row>
-    <row r="3" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>65</v>
       </c>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="D3" s="20"/>
     </row>
-    <row r="4" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>65</v>
       </c>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="D4" s="20"/>
     </row>
-    <row r="5" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
         <v>65</v>
       </c>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="D5" s="20"/>
     </row>
-    <row r="6" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>65</v>
       </c>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="D6" s="20"/>
     </row>
-    <row r="7" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>65</v>
       </c>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="D7" s="20"/>
     </row>
-    <row r="8" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>65</v>
       </c>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="D8" s="20"/>
     </row>
-    <row r="9" spans="1:16384" s="24" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16384" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
         <v>66</v>
       </c>
@@ -19717,7 +19717,7 @@
       <c r="XFC9" s="20"/>
       <c r="XFD9" s="20"/>
     </row>
-    <row r="10" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>66</v>
       </c>
@@ -19729,7 +19729,7 @@
       </c>
       <c r="D10" s="20"/>
     </row>
-    <row r="11" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>66</v>
       </c>
@@ -19741,7 +19741,7 @@
       </c>
       <c r="D11" s="20"/>
     </row>
-    <row r="12" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>66</v>
       </c>
@@ -19753,7 +19753,7 @@
       </c>
       <c r="D12" s="20"/>
     </row>
-    <row r="13" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>66</v>
       </c>
@@ -19765,7 +19765,7 @@
       </c>
       <c r="D13" s="20"/>
     </row>
-    <row r="14" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>66</v>
       </c>
@@ -19777,7 +19777,7 @@
       </c>
       <c r="D14" s="20"/>
     </row>
-    <row r="15" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>66</v>
       </c>
@@ -19789,7 +19789,7 @@
       </c>
       <c r="D15" s="20"/>
     </row>
-    <row r="16" spans="1:16384" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>66</v>
       </c>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="D16" s="20"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>66</v>
       </c>
@@ -19813,7 +19813,7 @@
       </c>
       <c r="D17" s="20"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="22" t="s">
         <v>67</v>
       </c>
@@ -19821,7 +19821,7 @@
       <c r="C18" s="23"/>
       <c r="D18" s="20"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>67</v>
       </c>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="D19" s="20"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>67</v>
       </c>
@@ -19845,7 +19845,7 @@
       </c>
       <c r="D20" s="20"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>67</v>
       </c>
@@ -19857,7 +19857,7 @@
       </c>
       <c r="D21" s="20"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>67</v>
       </c>
@@ -19869,7 +19869,7 @@
       </c>
       <c r="D22" s="20"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>67</v>
       </c>
@@ -19881,7 +19881,7 @@
       </c>
       <c r="D23" s="20"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>67</v>
       </c>
@@ -19893,7 +19893,7 @@
       </c>
       <c r="D24" s="20"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>67</v>
       </c>
@@ -19905,7 +19905,7 @@
       </c>
       <c r="D25" s="20"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>67</v>
       </c>
@@ -19917,7 +19917,7 @@
       </c>
       <c r="D26" s="20"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>67</v>
       </c>
@@ -19929,7 +19929,7 @@
       </c>
       <c r="D27" s="20"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
         <v>67</v>
       </c>
@@ -19941,7 +19941,7 @@
       </c>
       <c r="D28" s="20"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>67</v>
       </c>
@@ -19953,7 +19953,7 @@
       </c>
       <c r="D29" s="20"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
         <v>67</v>
       </c>
@@ -19965,7 +19965,7 @@
       </c>
       <c r="D30" s="20"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>67</v>
       </c>
@@ -19977,7 +19977,7 @@
       </c>
       <c r="D31" s="20"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
         <v>67</v>
       </c>
@@ -19989,7 +19989,7 @@
       </c>
       <c r="D32" s="20"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="22" t="s">
         <v>68</v>
       </c>
@@ -19997,7 +19997,7 @@
       <c r="C33" s="23"/>
       <c r="D33" s="20"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>68</v>
       </c>
@@ -20009,7 +20009,7 @@
       </c>
       <c r="D34" s="20"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="19" t="s">
         <v>68</v>
       </c>
@@ -20021,7 +20021,7 @@
       </c>
       <c r="D35" s="20"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
         <v>68</v>
       </c>
@@ -20033,7 +20033,7 @@
       </c>
       <c r="D36" s="20"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
         <v>68</v>
       </c>
@@ -20045,7 +20045,7 @@
       </c>
       <c r="D37" s="20"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
         <v>68</v>
       </c>
@@ -20057,7 +20057,7 @@
       </c>
       <c r="D38" s="20"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
         <v>68</v>
       </c>
@@ -20069,7 +20069,7 @@
       </c>
       <c r="D39" s="20"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>68</v>
       </c>
@@ -20081,7 +20081,7 @@
       </c>
       <c r="D40" s="20"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
         <v>68</v>
       </c>
@@ -20093,7 +20093,7 @@
       </c>
       <c r="D41" s="20"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="19" t="s">
         <v>68</v>
       </c>
@@ -20105,7 +20105,7 @@
       </c>
       <c r="D42" s="20"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>68</v>
       </c>
@@ -20117,7 +20117,7 @@
       </c>
       <c r="D43" s="20"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="19" t="s">
         <v>68</v>
       </c>
@@ -20129,7 +20129,7 @@
       </c>
       <c r="D44" s="20"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="19" t="s">
         <v>68</v>
       </c>
@@ -20141,7 +20141,7 @@
       </c>
       <c r="D45" s="20"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="19" t="s">
         <v>68</v>
       </c>
@@ -20153,7 +20153,7 @@
       </c>
       <c r="D46" s="20"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="19" t="s">
         <v>68</v>
       </c>
@@ -20165,7 +20165,7 @@
       </c>
       <c r="D47" s="20"/>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
         <v>68</v>
       </c>
@@ -20177,7 +20177,7 @@
       </c>
       <c r="D48" s="20"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="19" t="s">
         <v>68</v>
       </c>
@@ -20189,7 +20189,7 @@
       </c>
       <c r="D49" s="20"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="22" t="s">
         <v>69</v>
       </c>
@@ -20197,7 +20197,7 @@
       <c r="C50" s="23"/>
       <c r="D50" s="20"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="19" t="s">
         <v>69</v>
       </c>
@@ -20209,7 +20209,7 @@
       </c>
       <c r="D51" s="20"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="19" t="s">
         <v>69</v>
       </c>
@@ -20221,7 +20221,7 @@
       </c>
       <c r="D52" s="20"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="19" t="s">
         <v>69</v>
       </c>
@@ -20233,7 +20233,7 @@
       </c>
       <c r="D53" s="20"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="19" t="s">
         <v>69</v>
       </c>
@@ -20245,7 +20245,7 @@
       </c>
       <c r="D54" s="20"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="19" t="s">
         <v>69</v>
       </c>
@@ -20257,7 +20257,7 @@
       </c>
       <c r="D55" s="20"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="19" t="s">
         <v>69</v>
       </c>
@@ -20269,7 +20269,7 @@
       </c>
       <c r="D56" s="20"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="19" t="s">
         <v>69</v>
       </c>
@@ -20281,7 +20281,7 @@
       </c>
       <c r="D57" s="20"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="22" t="s">
         <v>70</v>
       </c>
@@ -20289,7 +20289,7 @@
       <c r="C58" s="23"/>
       <c r="D58" s="20"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="19" t="s">
         <v>70</v>
       </c>
@@ -20301,7 +20301,7 @@
       </c>
       <c r="D59" s="20"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="19" t="s">
         <v>70</v>
       </c>
@@ -20313,7 +20313,7 @@
       </c>
       <c r="D60" s="20"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="19" t="s">
         <v>70</v>
       </c>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="D61" s="20"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="19" t="s">
         <v>70</v>
       </c>
@@ -20337,7 +20337,7 @@
       </c>
       <c r="D62" s="20"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="19" t="s">
         <v>70</v>
       </c>
@@ -20349,7 +20349,7 @@
       </c>
       <c r="D63" s="20"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="19" t="s">
         <v>70</v>
       </c>
@@ -20361,7 +20361,7 @@
       </c>
       <c r="D64" s="20"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="19" t="s">
         <v>70</v>
       </c>
@@ -20373,7 +20373,7 @@
       </c>
       <c r="D65" s="20"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="19" t="s">
         <v>70</v>
       </c>
@@ -20385,7 +20385,7 @@
       </c>
       <c r="D66" s="20"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="19" t="s">
         <v>70</v>
       </c>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="D67" s="20"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="19" t="s">
         <v>70</v>
       </c>
@@ -20409,7 +20409,7 @@
       </c>
       <c r="D68" s="20"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="19" t="s">
         <v>70</v>
       </c>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="D69" s="20"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="19" t="s">
         <v>70</v>
       </c>
@@ -20433,7 +20433,7 @@
       </c>
       <c r="D70" s="20"/>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="19" t="s">
         <v>70</v>
       </c>
@@ -20445,7 +20445,7 @@
       </c>
       <c r="D71" s="20"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="19" t="s">
         <v>70</v>
       </c>
@@ -20457,7 +20457,7 @@
       </c>
       <c r="D72" s="20"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="19" t="s">
         <v>70</v>
       </c>
@@ -20469,7 +20469,7 @@
       </c>
       <c r="D73" s="20"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="19" t="s">
         <v>70</v>
       </c>
@@ -20481,7 +20481,7 @@
       </c>
       <c r="D74" s="20"/>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="19" t="s">
         <v>70</v>
       </c>
@@ -20493,7 +20493,7 @@
       </c>
       <c r="D75" s="20"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
         <v>72</v>
       </c>
@@ -20501,7 +20501,7 @@
       <c r="C76" s="23"/>
       <c r="D76" s="20"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="19" t="s">
         <v>72</v>
       </c>
@@ -20513,7 +20513,7 @@
       </c>
       <c r="D77" s="20"/>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="19" t="s">
         <v>72</v>
       </c>
@@ -20525,7 +20525,7 @@
       </c>
       <c r="D78" s="20"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="19" t="s">
         <v>72</v>
       </c>
@@ -20537,7 +20537,7 @@
       </c>
       <c r="D79" s="20"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="19" t="s">
         <v>72</v>
       </c>
@@ -20549,7 +20549,7 @@
       </c>
       <c r="D80" s="20"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="19" t="s">
         <v>72</v>
       </c>
@@ -20561,7 +20561,7 @@
       </c>
       <c r="D81" s="20"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="19" t="s">
         <v>72</v>
       </c>
@@ -20573,7 +20573,7 @@
       </c>
       <c r="D82" s="20"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="19" t="s">
         <v>72</v>
       </c>
@@ -20585,7 +20585,7 @@
       </c>
       <c r="D83" s="20"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="19" t="s">
         <v>72</v>
       </c>
@@ -20597,7 +20597,7 @@
       </c>
       <c r="D84" s="20"/>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
         <v>73</v>
       </c>
@@ -20605,7 +20605,7 @@
       <c r="C85" s="23"/>
       <c r="D85" s="20"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="19" t="s">
         <v>73</v>
       </c>
@@ -20617,7 +20617,7 @@
       </c>
       <c r="D86" s="20"/>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="19" t="s">
         <v>73</v>
       </c>
@@ -20629,7 +20629,7 @@
       </c>
       <c r="D87" s="20"/>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="19" t="s">
         <v>73</v>
       </c>
@@ -20641,7 +20641,7 @@
       </c>
       <c r="D88" s="20"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="19" t="s">
         <v>73</v>
       </c>
@@ -20653,7 +20653,7 @@
       </c>
       <c r="D89" s="20"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="19" t="s">
         <v>73</v>
       </c>
@@ -20665,7 +20665,7 @@
       </c>
       <c r="D90" s="20"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="19" t="s">
         <v>73</v>
       </c>
@@ -20677,7 +20677,7 @@
       </c>
       <c r="D91" s="20"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="19" t="s">
         <v>73</v>
       </c>
@@ -20689,7 +20689,7 @@
       </c>
       <c r="D92" s="20"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="19" t="s">
         <v>73</v>
       </c>
@@ -20701,7 +20701,7 @@
       </c>
       <c r="D93" s="20"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="19" t="s">
         <v>73</v>
       </c>
@@ -20713,7 +20713,7 @@
       </c>
       <c r="D94" s="20"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="19" t="s">
         <v>73</v>
       </c>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="D95" s="20"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="19" t="s">
         <v>73</v>
       </c>
@@ -20737,7 +20737,7 @@
       </c>
       <c r="D96" s="20"/>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="19" t="s">
         <v>73</v>
       </c>
@@ -20749,7 +20749,7 @@
       </c>
       <c r="D97" s="20"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="22" t="s">
         <v>74</v>
       </c>
@@ -20757,7 +20757,7 @@
       <c r="C98" s="23"/>
       <c r="D98" s="20"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="19" t="s">
         <v>74</v>
       </c>
@@ -20769,7 +20769,7 @@
       </c>
       <c r="D99" s="20"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="19" t="s">
         <v>74</v>
       </c>
@@ -20781,7 +20781,7 @@
       </c>
       <c r="D100" s="20"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="19" t="s">
         <v>74</v>
       </c>
@@ -20793,7 +20793,7 @@
       </c>
       <c r="D101" s="20"/>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="19" t="s">
         <v>74</v>
       </c>
@@ -20805,7 +20805,7 @@
       </c>
       <c r="D102" s="20"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="19" t="s">
         <v>74</v>
       </c>
@@ -20817,7 +20817,7 @@
       </c>
       <c r="D103" s="20"/>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="19" t="s">
         <v>74</v>
       </c>
@@ -20829,7 +20829,7 @@
       </c>
       <c r="D104" s="20"/>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="19" t="s">
         <v>74</v>
       </c>
@@ -20841,7 +20841,7 @@
       </c>
       <c r="D105" s="20"/>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="25" t="s">
         <v>75</v>
       </c>
@@ -20849,7 +20849,7 @@
       <c r="C106" s="23"/>
       <c r="D106" s="20"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="19" t="s">
         <v>75</v>
       </c>
@@ -20861,7 +20861,7 @@
       </c>
       <c r="D107" s="20"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="19" t="s">
         <v>75</v>
       </c>
@@ -20873,7 +20873,7 @@
       </c>
       <c r="D108" s="20"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="19" t="s">
         <v>75</v>
       </c>
@@ -20885,7 +20885,7 @@
       </c>
       <c r="D109" s="20"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="19" t="s">
         <v>75</v>
       </c>
@@ -20897,7 +20897,7 @@
       </c>
       <c r="D110" s="20"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="19" t="s">
         <v>75</v>
       </c>
@@ -20909,7 +20909,7 @@
       </c>
       <c r="D111" s="20"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="19" t="s">
         <v>75</v>
       </c>
@@ -20921,7 +20921,7 @@
       </c>
       <c r="D112" s="20"/>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="19" t="s">
         <v>75</v>
       </c>
@@ -20933,7 +20933,7 @@
       </c>
       <c r="D113" s="20"/>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="22" t="s">
         <v>76</v>
       </c>
@@ -20941,7 +20941,7 @@
       <c r="C114" s="23"/>
       <c r="D114" s="20"/>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="19" t="s">
         <v>76</v>
       </c>
@@ -20953,7 +20953,7 @@
       </c>
       <c r="D115" s="20"/>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="19" t="s">
         <v>76</v>
       </c>
@@ -20965,7 +20965,7 @@
       </c>
       <c r="D116" s="20"/>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="19" t="s">
         <v>76</v>
       </c>
@@ -20977,7 +20977,7 @@
       </c>
       <c r="D117" s="20"/>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="19" t="s">
         <v>76</v>
       </c>
@@ -20989,7 +20989,7 @@
       </c>
       <c r="D118" s="20"/>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="19" t="s">
         <v>76</v>
       </c>
@@ -21001,14 +21001,14 @@
       </c>
       <c r="D119" s="20"/>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="22" t="s">
         <v>177</v>
       </c>
       <c r="B120" s="23"/>
       <c r="C120" s="23"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="19" t="s">
         <v>177</v>
       </c>
@@ -21019,7 +21019,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="19" t="s">
         <v>177</v>
       </c>
@@ -21039,24 +21039,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF5C93B5-7466-44B3-AFB0-A5F8BD24E813}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>180</v>
       </c>
@@ -21064,12 +21064,12 @@
         <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C6" s="27" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>185</v>
       </c>
@@ -21087,7 +21087,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>184</v>
       </c>
@@ -21095,12 +21095,12 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>189</v>
       </c>
@@ -21108,7 +21108,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>191</v>
       </c>
@@ -21119,7 +21119,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>191</v>
       </c>
@@ -21130,7 +21130,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>187</v>
       </c>
@@ -21138,7 +21138,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>193</v>
       </c>
@@ -21146,17 +21146,17 @@
         <v>195</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>200</v>
       </c>
@@ -21165,7 +21165,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>199</v>
       </c>
@@ -21174,7 +21174,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>201</v>
       </c>

</xml_diff>